<commit_message>
working code on 24th
Added - resource forecasting + Rule based notifications + updated alot in user and configuration
</commit_message>
<xml_diff>
--- a/Ref docs/Requests/Client Request Details.xlsx
+++ b/Ref docs/Requests/Client Request Details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/Requests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="434" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56AC4CC2-3C55-4C5D-B2BF-058A86024013}"/>
+  <xr:revisionPtr revIDLastSave="447" documentId="13_ncr:1_{CA1DD370-0662-49C9-B33F-52F3C5116C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD53684D-EA4F-4903-A99A-055C73B63192}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="63">
   <si>
     <t>Description</t>
   </si>
@@ -212,9 +212,6 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>15/01/2024</t>
-  </si>
-  <si>
     <t>ZS Onboarding Initiated</t>
   </si>
   <si>
@@ -279,9 +276,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-24009]m/d/yyyy;@"/>
-  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -369,7 +363,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -717,8 +711,7 @@
     <col min="3" max="3" width="42.6640625" style="5" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" style="5" customWidth="1"/>
     <col min="5" max="5" width="24" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.9140625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="11.83203125" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.9140625" style="7" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="8.6640625" style="5"/>
   </cols>
@@ -728,7 +721,7 @@
         <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -743,10 +736,10 @@
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -754,7 +747,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>18</v>
@@ -763,7 +756,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>2</v>
@@ -772,7 +765,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="8">
-        <v>45306</v>
+        <v>46037</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -780,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>19</v>
@@ -797,8 +790,8 @@
       <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>43</v>
+      <c r="H3" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -806,7 +799,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>20</v>
@@ -823,8 +816,8 @@
       <c r="G4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>43</v>
+      <c r="H4" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -832,7 +825,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>21</v>
@@ -849,8 +842,8 @@
       <c r="G5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>43</v>
+      <c r="H5" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -858,7 +851,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>22</v>
@@ -875,8 +868,8 @@
       <c r="G6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>43</v>
+      <c r="H6" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -884,7 +877,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>26</v>
@@ -901,8 +894,8 @@
       <c r="G7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>43</v>
+      <c r="H7" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -910,7 +903,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>27</v>
@@ -927,8 +920,8 @@
       <c r="G8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>43</v>
+      <c r="H8" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -936,7 +929,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>28</v>
@@ -945,7 +938,7 @@
         <v>11</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>34</v>
@@ -953,8 +946,8 @@
       <c r="G9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>43</v>
+      <c r="H9" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -962,7 +955,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>23</v>
@@ -979,8 +972,8 @@
       <c r="G10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>43</v>
+      <c r="H10" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -988,7 +981,7 @@
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>23</v>
@@ -997,7 +990,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>34</v>
@@ -1005,8 +998,8 @@
       <c r="G11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>43</v>
+      <c r="H11" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1014,7 +1007,7 @@
         <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>24</v>
@@ -1031,16 +1024,16 @@
       <c r="G12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>43</v>
+      <c r="H12" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>24</v>
@@ -1057,16 +1050,16 @@
       <c r="G13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>43</v>
+      <c r="H13" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>24</v>
@@ -1083,16 +1076,16 @@
       <c r="G14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>43</v>
+      <c r="H14" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>24</v>
@@ -1109,19 +1102,19 @@
       <c r="G15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>43</v>
+      <c r="H15" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>11</v>
@@ -1135,19 +1128,19 @@
       <c r="G16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>43</v>
+      <c r="H16" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>11</v>
@@ -1161,16 +1154,16 @@
       <c r="G17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>43</v>
+      <c r="H17" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>24</v>
@@ -1187,16 +1180,16 @@
       <c r="G18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>43</v>
+      <c r="H18" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>24</v>
@@ -1213,16 +1206,16 @@
       <c r="G19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>43</v>
+      <c r="H19" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>24</v>
@@ -1239,16 +1232,16 @@
       <c r="G20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>43</v>
+      <c r="H20" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>24</v>
@@ -1265,16 +1258,16 @@
       <c r="G21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>43</v>
+      <c r="H21" s="8">
+        <v>46037</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>24</v>
@@ -1291,8 +1284,8 @@
       <c r="G22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>43</v>
+      <c r="H22" s="8">
+        <v>45306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>